<commit_message>
Fix workbook intake bugs found against real 9.21.26 lists
Strip comma thousands separators in mileage, prefer Hogan O/S Status
over Photos label for completion, and allow reports.nationalinspect.com
inspection hosts so real Penske/Hogan workbooks preview and import cleanly.

Co-authored-by: mancavesports3024 <mancavesports3024@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/fixtures/sourcing/hogan-wholesale-sample.xlsx
+++ b/fixtures/sourcing/hogan-wholesale-sample.xlsx
@@ -463,7 +463,7 @@
         <v>192018</v>
       </c>
       <c r="C2" t="str">
-        <v>Not Started</v>
+        <v>Photos</v>
       </c>
       <c r="D2" t="str">
         <v>42000</v>
@@ -472,7 +472,7 @@
         <v>Wholesale</v>
       </c>
       <c r="F2" t="str">
-        <v>Available</v>
+        <v>Not Started</v>
       </c>
       <c r="G2" t="str">
         <v>31 - Kansas City, MO</v>

</xml_diff>